<commit_message>
Add Materials & Makes procurement tab with verified manufacturers
Deep-dive pass over the combined drawing set: full luminaire catalog
strings, complete TSY001 device schedule data (mounting heights, boxes,
conduit stubs), C-502/C-503 gate context (36' cantilever slide gates,
FE7 swing/personnel gates), and a new procurement tab with 30 items —
specified makes verified against product literature, basis-of-design
suggestions clearly marked, quantities live-linked to the takeoff tabs.
Adds RFI-13 (EB1 manufacturer discrepancy) and RFI-14 (incomplete
catalog strings).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFdSenHH5oJ8QjkasHPHCm
</commit_message>
<xml_diff>
--- a/DOE_GJ_Site_Improvement_Exterior_Elec_Comm_Takeoff.xlsx
+++ b/DOE_GJ_Site_Improvement_Exterior_Elec_Comm_Takeoff.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Site Electrical" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Telecom OSP" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Security" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Assumptions" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Materials &amp; Makes" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Assumptions" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="699">
   <si>
     <t xml:space="preserve">DETAILED QUANTITY TAKEOFF — EXTERIOR ELECTRICAL &amp; COMMUNICATIONS</t>
   </si>
@@ -545,16 +546,16 @@
     <t xml:space="preserve">C6</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixture EB1 — exterior LED bollard, at grade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">277V; 3000K, 80 CRI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luminis RADB-LED-P1-30K-SYM-PIR-BTT-BCF-HXX-DDXX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 bollards along Bldg A south walk; integral PIR.</t>
+    <t xml:space="preserve">Fixture EB1 — exterior LED bollard (RADEAN), at grade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8-1/4" dia x 41-1/2" H; 277V; 3000K, 80 CRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RADB-LED-P1-30K-SYM-PIR-BTT-BCF-HXX-DDXX (schedule lists 'Luminis'; RADB is a Lithonia/Acuity RADEAN model — see RFI-13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 bollards along Bldg A south walk; integral PIR, symmetric distribution.</t>
   </si>
   <si>
     <t xml:space="preserve">C7</t>
@@ -578,13 +579,13 @@
     <t xml:space="preserve">C8</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixture EF1 — exterior flagpole light, truck (trunnion) mounted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remote-driver LED; 3000K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eagle Mountain SG-3K-EHS-M-XX</t>
+    <t xml:space="preserve">Fixture EF1 — exterior flagpole downlight, truck mounted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size M (flags to 15'x25'); 3000K; remote driver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eagle Mountain Flag &amp; Flagpole 'StarGazer' SG-3K-EHS-M-XX (external-halyard stationary truck, dark-sky downlight)</t>
   </si>
   <si>
     <t xml:space="preserve">3 at flagpoles NW of Bldg A. Schedule voltage column shows 0V at 65% — driver remote (see C9).</t>
@@ -1295,6 +1296,555 @@
     <t xml:space="preserve">SECURITY TOTAL</t>
   </si>
   <si>
+    <t xml:space="preserve">MATERIALS, MAKES &amp; MODELS — PROCUREMENT LIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Specified' = named on the 65% drawings. 'Basis-of-design (suggested)' = drawings silent — a common product meeting the drawn requirements, offered for pricing only; Div 26/27/28 specs govern. Qty cells link live to the takeoff tabs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size / Rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model / Part No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spec Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIGHTING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area luminaire EA1 (Type 3, backlight control, house-side shield)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35' pole mt; 277V; 3000K/80CRI; P3 pkg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithonia Lighting (Acuity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSX1-LED-P3-30K-80CRI-BLC3-MVOLT-XXXX-PIR-SPD20KV-HS-EGSR-DDXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-Series Size 1. Wattage/lumen columns blank on 65% schedule — per fixture submittal. XXXX = distribution/finish fields to complete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area luminaire EA2 (Type 5 wide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSX1-LED-P3-30K-80CRI-T5W-MVOLT-XXXX-PIR-SPD20KV-EGSR-DDXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan symbol shows twin heads/pole — RFI-3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area luminaire EA3 (short-throw T1S, house-side shield)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSX1-LED-P3-30K-80CRI-T1S-MVOLT-XXXX-PIR-SPD20KV-HS-EGSR-DDXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Light pole, round straight steel or aluminum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35'-0 nominal; drilled for D-Series arm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valmont / RSA / Lithonia SSS (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per luminaire mfr pole selector, EPA per wind load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pole make/finish NOT scheduled at 65% — coordinate w/ luminaire order; anchor bolts per mfr (2/ES601).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED bollard EB1 (RADEAN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8-1/4" dia x 41-1/2" H; 277V; 3000K/80CRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithonia Lighting (Acuity) — schedule says 'Luminis'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RADB-LED-P1-30K-SYM-PIR-BTT-BCF-HXX-DDXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RADB is Lithonia's RADEAN bollard (Luminis is a sister Acuity brand) — RFI-13 to correct schedule mfr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flagpole downlight EF1 (StarGazer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size M (flags to 15'x25'); 3000K; LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eagle Mountain Flag &amp; Flagpole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG-3K-EHS-M-XX (external halyard, stationary truck)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dark-sky downlight; remote drivers in buried WP box (ES101 KN 10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WP enclosure for EF1 remote drivers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burial/landscape rated, NEMA 4/6P (assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD (per driver mfr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify enclosure &amp; driver model w/ Eagle Mountain submittal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERVICE &amp; POWER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pad-mount transformer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">480/277V 3-ph; kVA TBD by utility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xcel Energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By Others</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XE furnished/installed; pad &amp; grounding by GC/EC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meter housing + CT cabinet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per XE metering standard; NEMA 3R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milbank / B-Line (or per XE approved list)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per XE metering spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD (suggested)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC furnishes/installs housing; XE sets meter (ES101 KN 4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exterior JB for gate operator power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min 4-11/16" sq (NEC 314); NEMA 3R/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoffman / Wiegmann (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galvanized steel, gasketed, stamped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per ES101 KN 7; 2#10+1#10G, 3/4"C, 120V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ground rods &amp; bonding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5/8" x 8' (assumed); #6 bare Cu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERICO / Harger (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cu-clad rod + exothermic or irreversible compression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rod size not on drawings — confirm Div 26 spec.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TELECOM OSP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telecom maintenance hole MH1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8'-0" x 96" x 96"; base 9,275 lb / top 2,100 lb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oldcastle / Jensen Precast (or regional precaster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'4260' base + top deck per H1/TSN400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'4260' designation from detail — confirm precaster &amp; traffic rating of cover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telecom handhole HH1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hubbell/Quazite or Armorcast (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polymer concrete box + slip-resistant bolted cover, ANSI Tier (non-deliberate traffic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT vehicle-traffic rated per A1/TSN400 — keep out of pavement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duct bank conduit, 4"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4" PVC Type DB/EB (concrete-encased)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantex / JM Eagle (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB-60/DB-120 PVC duct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conduit-feet: DB1 LF x2 + DB2 LF x4 (live formula).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duct bank conduit, 2"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2" PVC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sch 40/DB PVC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB3 LF x 2 conduits (live formula).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabric innerduct, 4" 3-cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4", 3-cell, w/ pull tapes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxCell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxCell 4" 3-cell (MXE4 series)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'MaxCell' named on TSN100 duct bank schedule — one per conduit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabric innerduct, 2" 3-cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2", 3-cell, w/ pull tapes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxCell 2" 3-cell (MXE2 series)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One per DB3 conduit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSP fiber, 12-strand OM4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12F OM4 50/125 MM, OSP gel-free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corning / OFS (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e.g. Corning ALTOS 012TU4-T4790D20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type on TSN300 is generic '12-STRAND OM4 FIBER' — exact cable per Div 27 spec.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiber termination hardware @ Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12F LC (assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corning CCH / Panduit (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIU/patch panel + pigtails/splice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OTDR + IL testing per TIA; labeling per TIA-606.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detectable warning tape &amp; mule tape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6" tape @12" above duct; 1,250-lb tape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presco / Neptco (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"CAUTION BURIED TELECOM" + WP1250 mule tape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tape LF = trench LF (live).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECURITY (Div 28 — models per spec; BOD offered where drawings silent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video intercom door/pedestal station w/ integrated reader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PoE; vandal/weather resistant; flush or pedestal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aiphone (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IX Series 2 (e.g. IX-DVM) + reader module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches 'VIC' video intercom system &amp; extended-reach PoE copper architecture (TSY101).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Video intercom master station</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desktop, video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IX-MV7-* master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desktop mount per TSY001 schedule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gooseneck pedestal, 316 SS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48" above roadway; min 2" sq heavy wall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestal PRO (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">316 SS gooseneck w/ template L-bolts x4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welded 316 SS required by A1/TSY101; footer to frost +20" from curb.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card readers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mullion/single-gang; 3'-6" AFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HID (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signo 20 / 20K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reader tech (prox/SEOS/PIV) per DOE requirements — confirm; boxes per TSY001 schedule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access control panels ACP1/ACP2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surface mt 5'-0" AFF on fire-rated plywood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LenelS2 / Software House / Mercury-based (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per Div 28 spec &amp; DOE standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head-end platform not named on drawings — owner standard governs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gate position switch (DPS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industrial gate switch w/ armored lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sentrol/Edwards 2500-series (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e.g. 2507A w/ magnet &amp; bracket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per A7/TSY101: magnet on gate, switch on fence post, WP 1-gang box, 3/4"C to HH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle exit loops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preformed loop size per operator mfr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMX / Reno A&amp;E (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preformed loop + matching detector in operator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gate operators (36' cantilever slide gates per C-502/C-503) by others.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended-reach PoE copper data cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4-pair, 22 AWG min, OSP-rated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paige (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GameChanger PD2201EX (OSP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named performance (extended-reach, 22AWG, PoE) on TSY101/QC — GameChanger is the common BOD; verify E gate run length vs. mfr limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSP access control composite cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reader/lock/DPS/REX composite, OSP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Windy City Wire / West Penn (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per Div 28 spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment rack + SPDs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12U rack; SPDs on OSP copper &amp; device circuits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle Atlantic / CPI; DITEK (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12U wall rack; DTK series SPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rack per G2/TSY101; SPD line item Security B8.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASSUMPTIONS, CLARIFICATIONS &amp; EXCLUSIONS</t>
   </si>
   <si>
@@ -1539,6 +2089,39 @@
   </si>
   <si>
     <t xml:space="preserve">Confirm transformer kVA, generator kW/recertification requirements, and secondary conductor/conduit schedule (one-line, building package).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ES601 luminaire schedule lists EB1 manufacturer as 'Luminis', but model RADB-LED is Lithonia Lighting's RADEAN bollard (both Acuity brands) — confirm intended manufacturer/model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete the 'XXXX' placeholder fields in the DSX1 catalog strings (finish/options) and the blank wattage/lumen/CCT columns of the luminaire schedule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. MATERIALS &amp; MAKES TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 'Materials &amp; Makes' tab consolidates every product into a procurement list. 'Specified' items are named on the drawings (Lithonia DSX1 series, RADB/RADEAN bollard, Eagle Mountain StarGazer SG-EHS, MaxCell innerduct, '4260' precast MH). Where drawings are silent, a clearly-marked basis-of-design (BOD) suggestion is offered for pricing only — Div 26/27/28 specifications and DOE/owner standards govern final selection.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufacturer identities verified against current product literature: DSX1 = Lithonia D-Series Size 1 area luminaire (Acuity); RADB = Lithonia RADEAN bollard, 8-1/4" dia x 41-1/2" H (schedule's 'Luminis' appears to be an error — RFI-13); SG-3K-EHS-M = Eagle Mountain Flag &amp; Flagpole 'StarGazer' dark-sky flagpole downlight, external-halyard stationary truck, size M for flags to 15'x25'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qty cells on the Materials tab are live formulas linked to the takeoff tabs (green), including conduit-feet roll-ups (duct bank LF x conduits per bank). Changing a takeoff quantity updates the procurement list automatically.</t>
   </si>
 </sst>
 </file>
@@ -1677,7 +2260,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1711,13 +2294,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E2F3"/>
-        <bgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1770,7 +2359,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1919,6 +2508,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1980,7 +2581,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -3289,11 +3890,11 @@
         <v>171</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="26" t="s">
         <v>173</v>
       </c>
       <c r="C30" s="7" t="s">
@@ -3319,7 +3920,7 @@
         <f aca="false">IF(I30="","",G30*I30)</f>
         <v/>
       </c>
-      <c r="K30" s="8" t="s">
+      <c r="K30" s="27" t="s">
         <v>176</v>
       </c>
     </row>
@@ -3357,7 +3958,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
         <v>183</v>
       </c>
@@ -5710,7 +6311,1020 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:C52"/>
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <f aca="false">'Site Electrical'!G25</f>
+        <v>9</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G7" s="37" t="n">
+        <f aca="false">'Site Electrical'!G26</f>
+        <v>7</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
+        <v>442</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G8" s="37" t="n">
+        <f aca="false">'Site Electrical'!G27</f>
+        <v>2</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
+        <v>445</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G10" s="37" t="n">
+        <f aca="false">'Site Electrical'!G30</f>
+        <v>6</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>458</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G11" s="37" t="n">
+        <f aca="false">'Site Electrical'!G32</f>
+        <v>3</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="G12" s="37" t="n">
+        <f aca="false">'Site Electrical'!G33</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>469</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>470</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="34" t="s">
+        <v>474</v>
+      </c>
+      <c r="G14" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
+        <v>476</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="F15" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G15" s="37" t="n">
+        <f aca="false">'Site Electrical'!G20</f>
+        <v>1</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>483</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="F16" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G16" s="37" t="n">
+        <f aca="false">'Site Electrical'!G38</f>
+        <v>3</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
+        <v>489</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="F17" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G17" s="37" t="n">
+        <f aca="false">'Site Electrical'!G29</f>
+        <v>18</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>495</v>
+      </c>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="20"/>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>496</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="F19" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="G19" s="37" t="n">
+        <f aca="false">'Telecom OSP'!G6</f>
+        <v>4</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>502</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G20" s="37" t="n">
+        <f aca="false">'Telecom OSP'!G7</f>
+        <v>5</v>
+      </c>
+      <c r="H20" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="s">
+        <v>507</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>508</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="F21" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G21" s="37" t="n">
+        <f aca="false">ROUND('Telecom OSP'!G17*2+'Telecom OSP'!G20*4,0)</f>
+        <v>2499</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
+        <v>513</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G22" s="37" t="n">
+        <f aca="false">ROUND('Telecom OSP'!G23*2,0)</f>
+        <v>598</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
+        <v>518</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G23" s="37" t="n">
+        <f aca="false">ROUND('Telecom OSP'!G17*2+'Telecom OSP'!G20*4,0)</f>
+        <v>2499</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
+        <v>524</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>526</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="F24" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="G24" s="37" t="n">
+        <f aca="false">ROUND('Telecom OSP'!G23*2,0)</f>
+        <v>598</v>
+      </c>
+      <c r="H24" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
+        <v>529</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="F25" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G25" s="37" t="n">
+        <f aca="false">'Telecom OSP'!G34</f>
+        <v>1600</v>
+      </c>
+      <c r="H25" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
+        <v>535</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="F26" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G26" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
+        <v>541</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="F27" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G27" s="37" t="n">
+        <f aca="false">'Telecom OSP'!G26</f>
+        <v>1407</v>
+      </c>
+      <c r="H27" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>548</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>550</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="F29" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G29" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
+        <v>554</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>557</v>
+      </c>
+      <c r="F30" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G30" s="37" t="n">
+        <f aca="false">Security!G20</f>
+        <v>1</v>
+      </c>
+      <c r="H30" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
+        <v>559</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>560</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>562</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="F31" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G31" s="37" t="n">
+        <f aca="false">Security!G6</f>
+        <v>2</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21" t="s">
+        <v>565</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="F32" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G32" s="37" t="n">
+        <f aca="false">Security!G8+Security!G9</f>
+        <v>2</v>
+      </c>
+      <c r="H32" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
+        <v>571</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>572</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="G33" s="37" t="n">
+        <f aca="false">Security!G16+Security!G17</f>
+        <v>2</v>
+      </c>
+      <c r="H33" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>577</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="F34" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G34" s="37" t="n">
+        <f aca="false">Security!G12</f>
+        <v>3</v>
+      </c>
+      <c r="H34" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
+        <v>583</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>585</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="F35" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G35" s="37" t="n">
+        <f aca="false">Security!G11</f>
+        <v>3</v>
+      </c>
+      <c r="H35" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>589</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="F36" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G36" s="37" t="n">
+        <f aca="false">Security!G27</f>
+        <v>1400</v>
+      </c>
+      <c r="H36" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>595</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="F37" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G37" s="37" t="n">
+        <f aca="false">Security!G26</f>
+        <v>1800</v>
+      </c>
+      <c r="H37" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I37" s="8"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="s">
+        <v>600</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="F38" s="39" t="s">
+        <v>481</v>
+      </c>
+      <c r="G38" s="37" t="n">
+        <f aca="false">Security!G18</f>
+        <v>1</v>
+      </c>
+      <c r="H38" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>605</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:C59"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -5719,358 +7333,404 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="37" t="s">
-        <v>423</v>
+      <c r="B2" s="40" t="s">
+        <v>606</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="38" t="s">
-        <v>424</v>
-      </c>
-      <c r="C4" s="39"/>
+      <c r="B4" s="41" t="s">
+        <v>607</v>
+      </c>
+      <c r="C4" s="42"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="40" t="s">
-        <v>425</v>
+      <c r="B5" s="43" t="s">
+        <v>608</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>426</v>
+        <v>609</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="40" t="s">
-        <v>427</v>
+      <c r="B6" s="43" t="s">
+        <v>610</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>428</v>
+        <v>611</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="40" t="s">
-        <v>429</v>
+      <c r="B7" s="43" t="s">
+        <v>612</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>430</v>
+        <v>613</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="38" t="s">
-        <v>431</v>
-      </c>
-      <c r="C9" s="39"/>
+      <c r="B9" s="41" t="s">
+        <v>614</v>
+      </c>
+      <c r="C9" s="42"/>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="43" t="s">
         <v>76</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>432</v>
+        <v>615</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="43" t="s">
         <v>254</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>433</v>
+        <v>616</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="43" t="s">
         <v>60</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>434</v>
+        <v>617</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="43" t="s">
         <v>199</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>435</v>
+        <v>618</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="40" t="s">
-        <v>436</v>
+      <c r="B14" s="43" t="s">
+        <v>619</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>437</v>
+        <v>620</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="40" t="s">
-        <v>438</v>
+      <c r="B15" s="43" t="s">
+        <v>621</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>439</v>
+        <v>622</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="38" t="s">
-        <v>440</v>
-      </c>
-      <c r="C17" s="39"/>
+      <c r="B17" s="41" t="s">
+        <v>623</v>
+      </c>
+      <c r="C17" s="42"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="40" t="s">
-        <v>441</v>
+      <c r="B18" s="43" t="s">
+        <v>624</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>442</v>
+        <v>625</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="40" t="s">
-        <v>443</v>
+      <c r="B19" s="43" t="s">
+        <v>626</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>444</v>
+        <v>627</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="40" t="s">
-        <v>445</v>
+      <c r="B20" s="43" t="s">
+        <v>628</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>446</v>
+        <v>629</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="40" t="s">
-        <v>447</v>
+      <c r="B21" s="43" t="s">
+        <v>630</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>448</v>
+        <v>631</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="40" t="s">
-        <v>449</v>
+      <c r="B22" s="43" t="s">
+        <v>632</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>450</v>
+        <v>633</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="40" t="s">
-        <v>451</v>
+      <c r="B23" s="43" t="s">
+        <v>634</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>452</v>
+        <v>635</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="40" t="s">
-        <v>453</v>
+      <c r="B24" s="43" t="s">
+        <v>636</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>454</v>
+        <v>637</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="40" t="s">
-        <v>455</v>
+      <c r="B25" s="43" t="s">
+        <v>638</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>456</v>
+        <v>639</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="40" t="s">
-        <v>457</v>
+      <c r="B26" s="43" t="s">
+        <v>640</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>458</v>
+        <v>641</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="40" t="s">
-        <v>459</v>
+      <c r="B27" s="43" t="s">
+        <v>642</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>460</v>
+        <v>643</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="40" t="s">
-        <v>461</v>
+      <c r="B28" s="43" t="s">
+        <v>644</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>462</v>
+        <v>645</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="38" t="s">
-        <v>463</v>
-      </c>
-      <c r="C30" s="39"/>
+      <c r="B30" s="41" t="s">
+        <v>646</v>
+      </c>
+      <c r="C30" s="42"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="40" t="s">
-        <v>464</v>
+      <c r="B31" s="43" t="s">
+        <v>647</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>465</v>
+        <v>648</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="40" t="s">
-        <v>466</v>
+      <c r="B32" s="43" t="s">
+        <v>649</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>467</v>
+        <v>650</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="40" t="s">
-        <v>468</v>
+      <c r="B33" s="43" t="s">
+        <v>651</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>469</v>
+        <v>652</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="40" t="s">
-        <v>470</v>
+      <c r="B34" s="43" t="s">
+        <v>653</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>471</v>
+        <v>654</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="40" t="s">
-        <v>472</v>
+      <c r="B35" s="43" t="s">
+        <v>655</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>473</v>
+        <v>656</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="40" t="s">
-        <v>474</v>
+      <c r="B36" s="43" t="s">
+        <v>657</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>475</v>
+        <v>658</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="40" t="s">
-        <v>476</v>
+      <c r="B37" s="43" t="s">
+        <v>659</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>477</v>
+        <v>660</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="40" t="s">
-        <v>478</v>
+      <c r="B38" s="43" t="s">
+        <v>661</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>479</v>
+        <v>662</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="38" t="s">
-        <v>480</v>
-      </c>
-      <c r="C40" s="39"/>
+      <c r="B40" s="41" t="s">
+        <v>663</v>
+      </c>
+      <c r="C40" s="42"/>
     </row>
     <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="40" t="s">
-        <v>481</v>
+      <c r="B41" s="43" t="s">
+        <v>664</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>482</v>
+        <v>665</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="40" t="s">
-        <v>483</v>
+      <c r="B42" s="43" t="s">
+        <v>666</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>484</v>
+        <v>667</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="40" t="s">
-        <v>485</v>
+      <c r="B43" s="43" t="s">
+        <v>668</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>486</v>
+        <v>669</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="40" t="s">
-        <v>487</v>
+      <c r="B44" s="43" t="s">
+        <v>670</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>488</v>
+        <v>671</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="40" t="s">
-        <v>489</v>
+      <c r="B45" s="43" t="s">
+        <v>672</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>490</v>
+        <v>673</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="40" t="s">
-        <v>491</v>
+      <c r="B46" s="43" t="s">
+        <v>674</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>492</v>
+        <v>675</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="40" t="s">
-        <v>493</v>
+      <c r="B47" s="43" t="s">
+        <v>676</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>494</v>
+        <v>677</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="40" t="s">
-        <v>495</v>
+      <c r="B48" s="43" t="s">
+        <v>678</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>496</v>
+        <v>679</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="40" t="s">
-        <v>497</v>
+      <c r="B49" s="43" t="s">
+        <v>680</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>498</v>
+        <v>681</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="40" t="s">
-        <v>499</v>
+      <c r="B50" s="43" t="s">
+        <v>682</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>500</v>
+        <v>683</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="40" t="s">
-        <v>501</v>
+      <c r="B51" s="43" t="s">
+        <v>684</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>502</v>
+        <v>685</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="40" t="s">
-        <v>503</v>
+      <c r="B52" s="43" t="s">
+        <v>686</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>504</v>
+        <v>687</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="43" t="s">
+        <v>688</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="43" t="s">
+        <v>690</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="41" t="s">
+        <v>692</v>
+      </c>
+      <c r="C56" s="42"/>
+    </row>
+    <row r="57" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B57" s="43" t="s">
+        <v>693</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="43" t="s">
+        <v>695</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B59" s="43" t="s">
+        <v>697</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Cable Schedule tab: run-by-run wire and conduit counts
New tab builds every security and comm cable run over its actual MH/HH
path with live lengths from the TSN100 segments plus adjustable interior
and slack inputs: 5 ACS runs (1,993 LF), 3 extended-reach data runs
(1,209 LF), 3 DPS runs (1,209 LF), 3 fiber runs with coils (1,425 LF).
Device conduit stubs itemized (7x 1" / 140 LF, 5x 3/4" / 85 LF) and a
duct bank occupancy matrix shows cables per segment vs. MaxCell cells.
Takeoff and procurement quantities now link to these totals.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HFdSenHH5oJ8QjkasHPHCm
</commit_message>
<xml_diff>
--- a/DOE_GJ_Site_Improvement_Exterior_Elec_Comm_Takeoff.xlsx
+++ b/DOE_GJ_Site_Improvement_Exterior_Elec_Comm_Takeoff.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Site Electrical" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Telecom OSP" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Security" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Materials &amp; Makes" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Assumptions" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Cable Schedule" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Materials &amp; Makes" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Assumptions" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1167" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1337" uniqueCount="893">
   <si>
     <t xml:space="preserve">DETAILED QUANTITY TAKEOFF — EXTERIOR ELECTRICAL &amp; COMMUNICATIONS</t>
   </si>
@@ -1095,7 +1096,7 @@
     <t xml:space="preserve">D. OSP CABLING (TSN300 site one-line)</t>
   </si>
   <si>
-    <t xml:space="preserve">OSP fiber — Bldg A to MH/HH system incl. coils for future connection at Bldg B/C and east gate handholes</t>
+    <t xml:space="preserve">OSP fiber — Bldg A to MH/HH system incl. coils for future connection at Bldg B/C and east gate handholes (3 runs)</t>
   </si>
   <si>
     <t xml:space="preserve">12-strand</t>
@@ -1104,10 +1105,10 @@
     <t xml:space="preserve">OM4 50/125 multimode, OSP-rated (gel-free, assumed), green-dashed runs per TSN300</t>
   </si>
   <si>
-    <t xml:space="preserve">TSN300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Routes + 20% slack + coils (QC: coiled for future connection at HH1s). Revise when cable schedule issued.</t>
+    <t xml:space="preserve">TSN300; Cable Schedule F1-F3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run-by-run buildup on Cable Schedule tab (segments + coil + interior + slack). QC: fiber coiled for future connection at HH1s.</t>
   </si>
   <si>
     <t xml:space="preserve">Fiber terminations, LIU/patch panel at Bldg A, testing &amp; documentation</t>
@@ -1356,22 +1357,22 @@
     <t xml:space="preserve">C. CABLING (homeruns via telecom duct bank system to COMM 124)</t>
   </si>
   <si>
-    <t xml:space="preserve">OSP-rated access control cable to each card reader location</t>
+    <t xml:space="preserve">OSP-rated access control cable to each card reader location (5 runs)</t>
   </si>
   <si>
     <t xml:space="preserve">Composite/multi-conductor per spec 28</t>
   </si>
   <si>
-    <t xml:space="preserve">OSP-rated ACS cable (reader/lock/DPS/REX composite assumed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSY100 QC notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 reader locations; homerun lengths estimated along duct routes + slack.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extended-reach copper data cable to each intercom (3)</t>
+    <t xml:space="preserve">OSP-rated ACS cable (reader/lock/REX composite assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSY100 QC; Cable Schedule R1-R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run-by-run buildup on Cable Schedule tab (path lengths live from TSN100 segments + interior &amp; slack inputs).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended-reach copper data cable to each intercom (3 runs)</t>
   </si>
   <si>
     <t xml:space="preserve">4-pair, 22 AWG min</t>
@@ -1380,10 +1381,10 @@
     <t xml:space="preserve">Extended-reach PoE-rated OSP copper data cable (per TSY101 riser note &amp; QC keynote)</t>
   </si>
   <si>
-    <t xml:space="preserve">TSY101; TSY100 QC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(3) cables per riser note. Verify length/bandwidth/PoE load/voltage-drop per mfr (GN 9) — east gate run ±600 LF.</t>
+    <t xml:space="preserve">TSY101; Cable Schedule R3-R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify length/bandwidth/PoE load/voltage-drop per mfr (GN 9) — east gate run ±560 LF vs. extended-reach limit.</t>
   </si>
   <si>
     <t xml:space="preserve">ACS cables, ACP1/ACP2 to Bldg A doors/monitored devices — BUILDING PACKAGE</t>
@@ -1401,6 +1402,51 @@
     <t xml:space="preserve">TSY002; TSY100 GN 8</t>
   </si>
   <si>
+    <t xml:space="preserve">Gate position switch (DPS) monitoring cable to head end (3 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-cond shielded OSP (assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSP-rated supervision pair per DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A7/TSY101; Cable Schedule R3-R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumes DPS monitored at ACP (not in operator) — verify signal path; if landed in operator, delete this line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device conduit stubs &amp; risers — 1"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1" (7 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PVC/RGS stub-ups: pedestal risers (2), bldg intercom stub (1), gate rough-ins (2)x1" x2 gates (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1,A13/TSY101; TSY001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Itemized on Cable Schedule Table C. Conduit described in device rows A1/A2/A8 is PRICED HERE ONLY — do not double-count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device conduit stubs — 3/4"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/4" (5 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PVC/RGS: reader stubs (2), DPS box-to-handhole (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A7/TSY101; TSY001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Itemized on Cable Schedule Table C; lengths assumed (heights/routing not dimensioned).</t>
+  </si>
+  <si>
     <t xml:space="preserve">D. EXCLUSIONS (struck from TSY002 responsibility matrix at 65% — VERIFY)</t>
   </si>
   <si>
@@ -1425,6 +1471,309 @@
     <t xml:space="preserve">SECURITY TOTAL</t>
   </si>
   <si>
+    <t xml:space="preserve">CABLE &amp; CONDUIT SCHEDULE — SECURITY &amp; COMMUNICATIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run lengths are LIVE: each path sums the TSN100 duct bank segments (Telecom OSP tab) + interior allowance, times (1 + slack). Adjust the yellow inputs and every cable total, takeoff line and procurement quantity follows.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPUTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interior allowance, duct bank entry to COMM 124 rack (per run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMM 124 location within Bldg A not shown in site set — verify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slack / service loops / vertical rises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiber coil at each future-connection handhole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLE A — SECURITY CABLE RUNS (homeruns to COMM 124, Bldg A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device / location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Path (via structures)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site path LF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run LF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestrian gate card reader @ Bldg C (HH1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-2 &gt; MH1-2 &gt; MH1-3 &gt; Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swing gate card reader (TSY101 inset — path assumed as R1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify vs. RFI-4 (possible overlap w/ R1 reader).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle gate 1 — Bldg B intercom/reader (HH1-4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-4 &gt; MH1-2 &gt; MH1-3 &gt; Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle gate 2 — pedestal @ HH1-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-5 &gt; HH1-3 &gt; MH1-4 &gt; MH1-3 &gt; Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle gate 3 — pedestal @ HH1-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-6 &gt; HH1-5 &gt; HH1-3 &gt; MH1-4 &gt; MH1-3 &gt; Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-ACS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACS cable total (5 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended-reach data total (3 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-DPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPS monitoring total (3 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLE B — COMM FIBER RUNS (12-strand OM4, TSN300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From &gt; To</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; HH1-2 (coil for future Bldg C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; MH1-3 &gt; MH1-2 &gt; HH1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; HH1-4 (coil for future Bldg B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; MH1-3 &gt; MH1-2 &gt; HH1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; HH1-6 (coil, east gates)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg A &gt; MH1-3 &gt; MH1-4 &gt; HH1-3 &gt; HH1-5 &gt; HH1-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-FIBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OM4 fiber total (3 runs incl. coils)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(info)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISP fiber, pedestal &gt; Bldg A — BY ISP (pathway only in contract)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISP ped &gt; MH1-1 &gt; MH1-2 &gt; MH1-3 &gt; Bldg A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLE C — DEVICE CONDUIT STUBS &amp; RISERS (security field devices; lengths assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conduit run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF ea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF tot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedestal riser, signal (A1/TSY101 detail — '1" conduit for signal cables')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bldg B intercom/reader stub to accessible ceiling (TSY001)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gate rough-in, (2) 1" conduits to SEC x 2 gates (A13/TSY101)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card reader stub (ped. &amp; swing gates, TSY001)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/4"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPS WP box to handhole (A7/TSY101)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-C1IN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total 1" device conduit (7 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOT-C34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total 3/4" device conduit (5 runs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLE D — DUCT BANK SEGMENT OCCUPANCY (cables riding each segment — info for pulling &amp; cell assignment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seg.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duct bank segment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cells</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-3 &gt; Bldg A entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heaviest segment — 14 cables in 12 cells; multiple LV cables per fabric cell is normal, but assign cells deliberately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-2 &gt; MH1-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-3 &gt; MH1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-4 &gt; HH1-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-3 &gt; HH1-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HH1-5 &gt; HH1-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-2 &gt; HH1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-2 &gt; HH1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-1 &gt; MH1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISP fiber only (by ISP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MH1-1 &gt; ISP pedestal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cells = conduits x 3 MaxCell cells. Counts are pass-through cables per this schedule's runs; ISP fiber (B1/B2/B8/B9) is pulled by ISP. No cables in vacant cells — plug per Telecom C11.</t>
+  </si>
+  <si>
     <t xml:space="preserve">MATERIALS, MAKES &amp; MODELS — PROCUREMENT LIST</t>
   </si>
   <si>
@@ -2059,6 +2408,24 @@
   </si>
   <si>
     <t xml:space="preserve">Rack per G2/TSY101; SPD line item Security B8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPS monitoring cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-cond shielded, OSP-rated (assumed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belden / West Penn (or equal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSP supervision pair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 runs per Cable Schedule; delete if DPS lands in gate operator instead of ACP.</t>
   </si>
   <si>
     <t xml:space="preserve">ASSUMPTIONS, CLARIFICATIONS &amp; EXCLUSIONS</t>
@@ -2344,14 +2711,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
+    <numFmt numFmtId="169" formatCode="0%"/>
+    <numFmt numFmtId="170" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2461,9 +2830,14 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF1F4E79"/>
+      <i val="true"/>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2471,6 +2845,14 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
+      <color rgb="FF1F4E79"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2575,7 +2957,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2720,12 +3102,72 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2736,7 +3178,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2748,7 +3190,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3091,7 +3533,7 @@
         <v>16</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">Security!J37</f>
+        <f aca="false">Security!J40</f>
         <v>0</v>
       </c>
       <c r="E11" s="8" t="s">
@@ -5673,10 +6115,11 @@
         <v>359</v>
       </c>
       <c r="F39" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="G39" s="22" t="n">
-        <v>1600</v>
+        <v>308</v>
+      </c>
+      <c r="G39" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-FIBER",'Cable Schedule'!A:A,0))</f>
+        <v>1425</v>
       </c>
       <c r="H39" s="21" t="s">
         <v>61</v>
@@ -5842,7 +6285,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -6440,7 +6883,7 @@
       <c r="H22" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="I22" s="36"/>
+      <c r="I22" s="37"/>
       <c r="J22" s="35"/>
       <c r="K22" s="27" t="s">
         <v>439</v>
@@ -6528,10 +6971,11 @@
         <v>446</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="G26" s="22" t="n">
-        <v>1800</v>
+        <v>308</v>
+      </c>
+      <c r="G26" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-ACS",'Cable Schedule'!A:A,0))</f>
+        <v>1993</v>
       </c>
       <c r="H26" s="21" t="s">
         <v>61</v>
@@ -6562,10 +7006,11 @@
         <v>451</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="G27" s="22" t="n">
-        <v>1400</v>
+        <v>308</v>
+      </c>
+      <c r="G27" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-DATA",'Cable Schedule'!A:A,0))</f>
+        <v>1209</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>61</v>
@@ -6604,7 +7049,7 @@
       <c r="H28" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="I28" s="36"/>
+      <c r="I28" s="37"/>
       <c r="J28" s="35"/>
       <c r="K28" s="8" t="s">
         <v>454</v>
@@ -6642,138 +7087,150 @@
       </c>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="30" t="n">
-        <f aca="false">SUM(J26:J29)</f>
-        <v>0</v>
-      </c>
-      <c r="K30" s="28"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="s">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B30" s="26" t="s">
         <v>458</v>
       </c>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
+      <c r="C30" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>461</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="G30" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-DPS",'Cable Schedule'!A:A,0))</f>
+        <v>1209</v>
+      </c>
+      <c r="H30" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I30" s="23"/>
+      <c r="J30" s="24" t="str">
+        <f aca="false">IF(I30="","",G30*I30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="27" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31" s="26" t="s">
+        <v>463</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>466</v>
+      </c>
+      <c r="F31" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="G31" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-C1IN",'Cable Schedule'!A:A,0))</f>
+        <v>140</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I31" s="23"/>
+      <c r="J31" s="24" t="str">
+        <f aca="false">IF(I31="","",G31*I31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="27" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>468</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="E32" s="21" t="s">
+        <v>471</v>
+      </c>
+      <c r="F32" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="G32" s="36" t="n">
+        <f aca="false">INDEX('Cable Schedule'!E:E,MATCH("TOT-C34",'Cable Schedule'!A:A,0))</f>
+        <v>85</v>
+      </c>
+      <c r="H32" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I32" s="23"/>
+      <c r="J32" s="24" t="str">
+        <f aca="false">IF(I32="","",G32*I32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="27" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="28"/>
+      <c r="B33" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="30" t="n">
+        <f aca="false">SUM(J26:J32)</f>
+        <v>0</v>
+      </c>
+      <c r="K33" s="28"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="s">
+        <v>473</v>
+      </c>
+      <c r="B34" s="20"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="20"/>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="B32" s="26" t="s">
-        <v>459</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>437</v>
-      </c>
-      <c r="F32" s="21" t="s">
-        <v>438</v>
-      </c>
-      <c r="G32" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="I32" s="36"/>
-      <c r="J32" s="35"/>
-      <c r="K32" s="27" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="s">
-        <v>226</v>
-      </c>
-      <c r="B33" s="26" t="s">
-        <v>461</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>437</v>
-      </c>
-      <c r="F33" s="21" t="s">
-        <v>438</v>
-      </c>
-      <c r="G33" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="I33" s="36"/>
-      <c r="J33" s="35"/>
-      <c r="K33" s="27" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
-        <v>231</v>
-      </c>
-      <c r="B34" s="26" t="s">
-        <v>462</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>437</v>
-      </c>
-      <c r="F34" s="21" t="s">
-        <v>438</v>
-      </c>
-      <c r="G34" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="I34" s="36"/>
-      <c r="J34" s="35"/>
-      <c r="K34" s="27" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="s">
-        <v>237</v>
-      </c>
       <c r="B35" s="26" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>65</v>
@@ -6793,29 +7250,122 @@
       <c r="H35" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="I35" s="36"/>
+      <c r="I35" s="37"/>
       <c r="J35" s="35"/>
       <c r="K35" s="27" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11"/>
-      <c r="B37" s="10" t="s">
-        <v>465</v>
-      </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="12" t="n">
-        <f aca="false">J14+J24+J30</f>
+        <v>475</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>476</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="F36" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="G36" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="11"/>
+      <c r="H36" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I36" s="37"/>
+      <c r="J36" s="35"/>
+      <c r="K36" s="27" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="s">
+        <v>231</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>477</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="G37" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I37" s="37"/>
+      <c r="J37" s="35"/>
+      <c r="K37" s="27" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" s="26" t="s">
+        <v>479</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E38" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="F38" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I38" s="37"/>
+      <c r="J38" s="35"/>
+      <c r="K38" s="27" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11"/>
+      <c r="B40" s="10" t="s">
+        <v>480</v>
+      </c>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="12" t="n">
+        <f aca="false">J14+J24+J33</f>
+        <v>0</v>
+      </c>
+      <c r="K40" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6833,7 +7383,1024 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="5" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="C5" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="C7" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="41" t="s">
+        <v>498</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B3",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>306.4</v>
+      </c>
+      <c r="E11" s="43" t="n">
+        <f aca="false">ROUND((D11+$C$5)*(1+$C$6),0)</f>
+        <v>392</v>
+      </c>
+      <c r="F11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="41" t="s">
+        <v>501</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>502</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="D12" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B3",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>306.4</v>
+      </c>
+      <c r="E12" s="43" t="n">
+        <f aca="false">ROUND((D12+$C$5)*(1+$C$6),0)</f>
+        <v>392</v>
+      </c>
+      <c r="F12" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="44"/>
+      <c r="J12" s="45" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="41" t="s">
+        <v>504</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D13" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B4",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>231.4</v>
+      </c>
+      <c r="E13" s="43" t="n">
+        <f aca="false">ROUND((D13+$C$5)*(1+$C$6),0)</f>
+        <v>310</v>
+      </c>
+      <c r="F13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="41" t="s">
+        <v>507</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="D14" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B11",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B6",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B5",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>259.7</v>
+      </c>
+      <c r="E14" s="43" t="n">
+        <f aca="false">ROUND((D14+$C$5)*(1+$C$6),0)</f>
+        <v>341</v>
+      </c>
+      <c r="F14" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="41" t="s">
+        <v>510</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>511</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="D15" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B12",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B11",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B6",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B5",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>457</v>
+      </c>
+      <c r="E15" s="43" t="n">
+        <f aca="false">ROUND((D15+$C$5)*(1+$C$6),0)</f>
+        <v>558</v>
+      </c>
+      <c r="F15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="29" t="s">
+        <v>513</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>514</v>
+      </c>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="46" t="n">
+        <f aca="false">SUMPRODUCT(E11:E15,F11:F15)</f>
+        <v>1993</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="29" t="s">
+        <v>515</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>516</v>
+      </c>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="46" t="n">
+        <f aca="false">SUMPRODUCT(E11:E15,G11:G15)</f>
+        <v>1209</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="28"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="29" t="s">
+        <v>517</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>518</v>
+      </c>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="46" t="n">
+        <f aca="false">SUMPRODUCT(E11:E15,H11:H15)</f>
+        <v>1209</v>
+      </c>
+      <c r="F18" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="41" t="s">
+        <v>521</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="D22" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B3",'Telecom OSP'!A:A,0))</f>
+        <v>306.4</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <f aca="false">ROUND((D22+$C$7+$C$5)*(1+$C$6),0)</f>
+        <v>447</v>
+      </c>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="44"/>
+      <c r="J22" s="44"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="41" t="s">
+        <v>524</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="D23" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B4",'Telecom OSP'!A:A,0))</f>
+        <v>231.4</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <f aca="false">ROUND((D23+$C$7+$C$5)*(1+$C$6),0)</f>
+        <v>365</v>
+      </c>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="44"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="41" t="s">
+        <v>527</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>529</v>
+      </c>
+      <c r="D24" s="42" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B5",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B6",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B11",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B12",'Telecom OSP'!A:A,0))</f>
+        <v>457</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <f aca="false">ROUND((D24+$C$7+$C$5)*(1+$C$6),0)</f>
+        <v>613</v>
+      </c>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="44"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="29" t="s">
+        <v>530</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>531</v>
+      </c>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="46" t="n">
+        <f aca="false">SUM(E22:E24)</f>
+        <v>1425</v>
+      </c>
+      <c r="F25" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="28"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D26" s="48" t="n">
+        <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("B1",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B2",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B8",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("B9",'Telecom OSP'!A:A,0))</f>
+        <v>716.4</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="41" t="s">
+        <v>541</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="C30" s="41" t="s">
+        <v>543</v>
+      </c>
+      <c r="D30" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="43" t="n">
+        <f aca="false">D30*E30</f>
+        <v>20</v>
+      </c>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="41" t="s">
+        <v>544</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C31" s="41" t="s">
+        <v>543</v>
+      </c>
+      <c r="D31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="F31" s="43" t="n">
+        <f aca="false">D31*E31</f>
+        <v>20</v>
+      </c>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="41" t="s">
+        <v>546</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="C32" s="41" t="s">
+        <v>543</v>
+      </c>
+      <c r="D32" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="F32" s="43" t="n">
+        <f aca="false">D32*E32</f>
+        <v>100</v>
+      </c>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="41" t="s">
+        <v>548</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>549</v>
+      </c>
+      <c r="C33" s="41" t="s">
+        <v>550</v>
+      </c>
+      <c r="D33" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="F33" s="43" t="n">
+        <f aca="false">D33*E33</f>
+        <v>40</v>
+      </c>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
+      <c r="J33" s="44"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="41" t="s">
+        <v>551</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C34" s="41" t="s">
+        <v>550</v>
+      </c>
+      <c r="D34" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="41" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" s="43" t="n">
+        <f aca="false">D34*E34</f>
+        <v>45</v>
+      </c>
+      <c r="G34" s="44"/>
+      <c r="H34" s="44"/>
+      <c r="I34" s="44"/>
+      <c r="J34" s="44"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="29" t="s">
+        <v>553</v>
+      </c>
+      <c r="B35" s="29" t="s">
+        <v>554</v>
+      </c>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="46" t="n">
+        <f aca="false">SUMPRODUCT((C30:C34="1""")*F30:F34)</f>
+        <v>140</v>
+      </c>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="28"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="29" t="s">
+        <v>555</v>
+      </c>
+      <c r="B36" s="29" t="s">
+        <v>556</v>
+      </c>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="46" t="n">
+        <f aca="false">SUMPRODUCT((C30:C34="3/4""")*F30:F34)</f>
+        <v>85</v>
+      </c>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="41" t="s">
+        <v>287</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="C40" s="41" t="s">
+        <v>566</v>
+      </c>
+      <c r="D40" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" s="49" t="n">
+        <f aca="false">SUM(D40:G40)</f>
+        <v>14</v>
+      </c>
+      <c r="I40" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="J40" s="50" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="41" t="s">
+        <v>284</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="C41" s="41" t="s">
+        <v>566</v>
+      </c>
+      <c r="D41" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="49" t="n">
+        <f aca="false">SUM(D41:G41)</f>
+        <v>7</v>
+      </c>
+      <c r="I41" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="J41" s="50"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="C42" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D42" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="49" t="n">
+        <f aca="false">SUM(D42:G42)</f>
+        <v>7</v>
+      </c>
+      <c r="I42" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J42" s="50"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="C43" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D43" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="49" t="n">
+        <f aca="false">SUM(D43:G43)</f>
+        <v>7</v>
+      </c>
+      <c r="I43" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J43" s="50"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="41" t="s">
+        <v>292</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="C44" s="41" t="s">
+        <v>573</v>
+      </c>
+      <c r="D44" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="49" t="n">
+        <f aca="false">SUM(D44:G44)</f>
+        <v>7</v>
+      </c>
+      <c r="I44" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J44" s="50"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="41" t="s">
+        <v>297</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="C45" s="41" t="s">
+        <v>573</v>
+      </c>
+      <c r="D45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="49" t="n">
+        <f aca="false">SUM(D45:G45)</f>
+        <v>4</v>
+      </c>
+      <c r="I45" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J45" s="50"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="41" t="s">
+        <v>128</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="C46" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D46" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="49" t="n">
+        <f aca="false">SUM(D46:G46)</f>
+        <v>3</v>
+      </c>
+      <c r="I46" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J46" s="50"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="C47" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D47" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="49" t="n">
+        <f aca="false">SUM(D47:G47)</f>
+        <v>4</v>
+      </c>
+      <c r="I47" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J47" s="50"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="41" t="s">
+        <v>123</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>577</v>
+      </c>
+      <c r="C48" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D48" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="49" t="n">
+        <f aca="false">SUM(D48:G48)</f>
+        <v>0</v>
+      </c>
+      <c r="I48" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J48" s="50" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>579</v>
+      </c>
+      <c r="C49" s="41" t="s">
+        <v>570</v>
+      </c>
+      <c r="D49" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="49" t="n">
+        <f aca="false">SUM(D49:G49)</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="J49" s="50" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="51" t="s">
+        <v>580</v>
+      </c>
+      <c r="B51" s="52" t="s">
+        <v>581</v>
+      </c>
+      <c r="C51" s="52"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="52"/>
+      <c r="F51" s="52"/>
+      <c r="G51" s="52"/>
+      <c r="H51" s="52"/>
+      <c r="I51" s="52"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B51:I51"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -6849,32 +8416,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>466</v>
+        <v>582</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>467</v>
+        <v>583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>468</v>
+        <v>584</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>469</v>
+        <v>585</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>470</v>
+        <v>586</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>471</v>
+        <v>587</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>472</v>
+        <v>588</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>50</v>
@@ -6888,7 +8455,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>473</v>
+        <v>589</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="20"/>
@@ -6901,24 +8468,24 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>474</v>
+        <v>590</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>475</v>
+        <v>591</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>476</v>
+        <v>592</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>477</v>
+        <v>593</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>478</v>
+        <v>594</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G6" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G6" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C1",'Site Electrical'!A:A,0))</f>
         <v>9</v>
       </c>
@@ -6926,29 +8493,29 @@
         <v>69</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>480</v>
+        <v>596</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>481</v>
+        <v>597</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>482</v>
+        <v>598</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>476</v>
+        <v>592</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>477</v>
+        <v>593</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>483</v>
+        <v>599</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G7" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G7" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C2",'Site Electrical'!A:A,0))</f>
         <v>7</v>
       </c>
@@ -6956,29 +8523,29 @@
         <v>69</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>484</v>
+        <v>600</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>485</v>
+        <v>601</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>486</v>
+        <v>602</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>476</v>
+        <v>592</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>477</v>
+        <v>593</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>487</v>
+        <v>603</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G8" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G8" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C3",'Site Electrical'!A:A,0))</f>
         <v>2</v>
       </c>
@@ -6989,24 +8556,24 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>488</v>
+        <v>604</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>489</v>
+        <v>605</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>490</v>
+        <v>606</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>491</v>
+        <v>607</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>492</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>493</v>
-      </c>
-      <c r="G9" s="37" t="n">
+        <v>608</v>
+      </c>
+      <c r="F9" s="53" t="s">
+        <v>609</v>
+      </c>
+      <c r="G9" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C4",'Site Electrical'!A:A,0))</f>
         <v>18</v>
       </c>
@@ -7014,29 +8581,29 @@
         <v>69</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>494</v>
+        <v>610</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>495</v>
+        <v>611</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>496</v>
+        <v>612</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>497</v>
+        <v>613</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>498</v>
+        <v>614</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>499</v>
+        <v>615</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G10" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G10" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C6",'Site Electrical'!A:A,0))</f>
         <v>6</v>
       </c>
@@ -7044,29 +8611,29 @@
         <v>69</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>500</v>
+        <v>616</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>501</v>
+        <v>617</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>502</v>
+        <v>618</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>503</v>
+        <v>619</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>504</v>
+        <v>620</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>505</v>
+        <v>621</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G11" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G11" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C8",'Site Electrical'!A:A,0))</f>
         <v>3</v>
       </c>
@@ -7074,29 +8641,29 @@
         <v>69</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>506</v>
+        <v>622</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>507</v>
+        <v>623</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>508</v>
+        <v>624</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>509</v>
+        <v>625</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>510</v>
+        <v>626</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="38" t="s">
-        <v>493</v>
-      </c>
-      <c r="G12" s="37" t="n">
+      <c r="F12" s="53" t="s">
+        <v>609</v>
+      </c>
+      <c r="G12" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C9",'Site Electrical'!A:A,0))</f>
         <v>1</v>
       </c>
@@ -7104,12 +8671,12 @@
         <v>69</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>511</v>
+        <v>627</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>512</v>
+        <v>628</v>
       </c>
       <c r="B13" s="20"/>
       <c r="C13" s="20"/>
@@ -7122,22 +8689,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>513</v>
+        <v>629</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>514</v>
+        <v>630</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>515</v>
+        <v>631</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>516</v>
+        <v>632</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>81</v>
       </c>
       <c r="F14" s="34" t="s">
-        <v>517</v>
+        <v>633</v>
       </c>
       <c r="G14" s="21" t="n">
         <v>1</v>
@@ -7146,29 +8713,29 @@
         <v>69</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>518</v>
+        <v>634</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>519</v>
+        <v>635</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>520</v>
+        <v>636</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>521</v>
+        <v>637</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>522</v>
+        <v>638</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>523</v>
-      </c>
-      <c r="F15" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G15" s="37" t="n">
+        <v>639</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G15" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("B3",'Site Electrical'!A:A,0))</f>
         <v>1</v>
       </c>
@@ -7176,29 +8743,29 @@
         <v>69</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>525</v>
+        <v>641</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>526</v>
+        <v>642</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>527</v>
+        <v>643</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>528</v>
+        <v>644</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>529</v>
+        <v>645</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>530</v>
-      </c>
-      <c r="F16" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G16" s="37" t="n">
+        <v>646</v>
+      </c>
+      <c r="F16" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G16" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("D1",'Site Electrical'!A:A,0))</f>
         <v>3</v>
       </c>
@@ -7206,29 +8773,29 @@
         <v>69</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>531</v>
+        <v>647</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>532</v>
+        <v>648</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>533</v>
+        <v>649</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>534</v>
+        <v>650</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>535</v>
+        <v>651</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>536</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G17" s="37" t="n">
+        <v>652</v>
+      </c>
+      <c r="F17" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G17" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C5",'Site Electrical'!A:A,0))</f>
         <v>18</v>
       </c>
@@ -7236,29 +8803,29 @@
         <v>69</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>537</v>
+        <v>653</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>538</v>
+        <v>654</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>539</v>
+        <v>655</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>540</v>
+        <v>656</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>541</v>
+        <v>657</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>542</v>
-      </c>
-      <c r="F18" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G18" s="37" t="n">
+        <v>658</v>
+      </c>
+      <c r="F18" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G18" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("D4",'Site Electrical'!A:A,0))</f>
         <v>3</v>
       </c>
@@ -7266,29 +8833,29 @@
         <v>69</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>543</v>
+        <v>659</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>544</v>
+        <v>660</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>545</v>
+        <v>661</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>233</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>546</v>
+        <v>662</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>547</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G19" s="37" t="n">
+        <v>663</v>
+      </c>
+      <c r="F19" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G19" s="36" t="n">
         <f aca="false">INDEX('Site Electrical'!G:G,MATCH("C12",'Site Electrical'!A:A,0))+INDEX('Site Electrical'!G:G,MATCH("D3",'Site Electrical'!A:A,0))</f>
         <v>56</v>
       </c>
@@ -7296,12 +8863,12 @@
         <v>69</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>548</v>
+        <v>664</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>549</v>
+        <v>665</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -7314,24 +8881,24 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>550</v>
+        <v>666</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>551</v>
+        <v>667</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>552</v>
+        <v>668</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>553</v>
+        <v>669</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>554</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>493</v>
-      </c>
-      <c r="G21" s="37" t="n">
+        <v>670</v>
+      </c>
+      <c r="F21" s="53" t="s">
+        <v>609</v>
+      </c>
+      <c r="G21" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("A1",'Telecom OSP'!A:A,0))</f>
         <v>4</v>
       </c>
@@ -7339,29 +8906,29 @@
         <v>69</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>555</v>
+        <v>671</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>556</v>
+        <v>672</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>557</v>
+        <v>673</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>257</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>558</v>
+        <v>674</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>559</v>
-      </c>
-      <c r="F22" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G22" s="37" t="n">
+        <v>675</v>
+      </c>
+      <c r="F22" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G22" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("A2",'Telecom OSP'!A:A,0))</f>
         <v>5</v>
       </c>
@@ -7369,29 +8936,29 @@
         <v>69</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>560</v>
+        <v>676</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>561</v>
+        <v>677</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>562</v>
+        <v>678</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>563</v>
+        <v>679</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>564</v>
+        <v>680</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>565</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G23" s="37" t="n">
+        <v>681</v>
+      </c>
+      <c r="F23" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G23" s="36" t="n">
         <f aca="false">ROUND(INDEX('Telecom OSP'!G:G,MATCH("B7",'Telecom OSP'!A:A,0))*2+INDEX('Telecom OSP'!G:G,MATCH("B10",'Telecom OSP'!A:A,0))*4,0)</f>
         <v>2499</v>
       </c>
@@ -7399,29 +8966,29 @@
         <v>61</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>566</v>
+        <v>682</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>567</v>
+        <v>683</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>568</v>
+        <v>684</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>569</v>
+        <v>685</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>564</v>
+        <v>680</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>570</v>
-      </c>
-      <c r="F24" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G24" s="37" t="n">
+        <v>686</v>
+      </c>
+      <c r="F24" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G24" s="36" t="n">
         <f aca="false">ROUND(INDEX('Telecom OSP'!G:G,MATCH("B13",'Telecom OSP'!A:A,0))*2,0)</f>
         <v>598</v>
       </c>
@@ -7429,29 +8996,29 @@
         <v>61</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>571</v>
+        <v>687</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>572</v>
+        <v>688</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>573</v>
+        <v>689</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>574</v>
+        <v>690</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>575</v>
+        <v>691</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>576</v>
+        <v>692</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G25" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G25" s="36" t="n">
         <f aca="false">ROUND(INDEX('Telecom OSP'!G:G,MATCH("B7",'Telecom OSP'!A:A,0))*2+INDEX('Telecom OSP'!G:G,MATCH("B10",'Telecom OSP'!A:A,0))*4,0)</f>
         <v>2499</v>
       </c>
@@ -7459,29 +9026,29 @@
         <v>61</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>577</v>
+        <v>693</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>578</v>
+        <v>694</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>579</v>
+        <v>695</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>580</v>
+        <v>696</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>575</v>
+        <v>691</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>581</v>
+        <v>697</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>479</v>
-      </c>
-      <c r="G26" s="37" t="n">
+        <v>595</v>
+      </c>
+      <c r="G26" s="36" t="n">
         <f aca="false">ROUND(INDEX('Telecom OSP'!G:G,MATCH("B13",'Telecom OSP'!A:A,0))*2,0)</f>
         <v>598</v>
       </c>
@@ -7489,57 +9056,57 @@
         <v>61</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>582</v>
+        <v>698</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>583</v>
+        <v>699</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>584</v>
+        <v>700</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>585</v>
+        <v>701</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>586</v>
+        <v>702</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>587</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G27" s="37" t="n">
+        <v>703</v>
+      </c>
+      <c r="F27" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G27" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("D1",'Telecom OSP'!A:A,0))</f>
-        <v>1600</v>
+        <v>1425</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>61</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>588</v>
+        <v>704</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>589</v>
+        <v>705</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>590</v>
+        <v>706</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>591</v>
+        <v>707</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>592</v>
+        <v>708</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>593</v>
-      </c>
-      <c r="F28" s="39" t="s">
-        <v>524</v>
+        <v>709</v>
+      </c>
+      <c r="F28" s="54" t="s">
+        <v>640</v>
       </c>
       <c r="G28" s="21" t="n">
         <v>1</v>
@@ -7548,29 +9115,29 @@
         <v>77</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>594</v>
+        <v>710</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>595</v>
+        <v>711</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>596</v>
+        <v>712</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>597</v>
+        <v>713</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>598</v>
+        <v>714</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>599</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G29" s="37" t="n">
+        <v>715</v>
+      </c>
+      <c r="F29" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G29" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("C1",'Telecom OSP'!A:A,0))</f>
         <v>1407</v>
       </c>
@@ -7578,29 +9145,29 @@
         <v>61</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>600</v>
+        <v>716</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>601</v>
+        <v>717</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>602</v>
+        <v>718</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>603</v>
+        <v>719</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>604</v>
+        <v>720</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>605</v>
-      </c>
-      <c r="F30" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G30" s="37" t="n">
+        <v>721</v>
+      </c>
+      <c r="F30" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G30" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("C7",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("C8",'Telecom OSP'!A:A,0))</f>
         <v>42</v>
       </c>
@@ -7608,29 +9175,29 @@
         <v>69</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>606</v>
+        <v>722</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>607</v>
+        <v>723</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>608</v>
+        <v>724</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>609</v>
+        <v>725</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>610</v>
+        <v>726</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>611</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G31" s="37" t="n">
+        <v>727</v>
+      </c>
+      <c r="F31" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G31" s="36" t="n">
         <f aca="false">INDEX('Telecom OSP'!G:G,MATCH("C9",'Telecom OSP'!A:A,0))+INDEX('Telecom OSP'!G:G,MATCH("C10",'Telecom OSP'!A:A,0))</f>
         <v>10</v>
       </c>
@@ -7638,27 +9205,27 @@
         <v>69</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>612</v>
+        <v>728</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>613</v>
+        <v>729</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>614</v>
+        <v>730</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>615</v>
+        <v>731</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>616</v>
+        <v>732</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>617</v>
-      </c>
-      <c r="F32" s="39" t="s">
-        <v>524</v>
+        <v>733</v>
+      </c>
+      <c r="F32" s="54" t="s">
+        <v>640</v>
       </c>
       <c r="G32" s="21" t="n">
         <v>1</v>
@@ -7667,12 +9234,12 @@
         <v>77</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>618</v>
+        <v>734</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>619</v>
+        <v>735</v>
       </c>
       <c r="B33" s="20"/>
       <c r="C33" s="20"/>
@@ -7685,22 +9252,22 @@
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>620</v>
+        <v>736</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>621</v>
+        <v>737</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>622</v>
+        <v>738</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>623</v>
+        <v>739</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="F34" s="39" t="s">
-        <v>524</v>
+        <v>740</v>
+      </c>
+      <c r="F34" s="54" t="s">
+        <v>640</v>
       </c>
       <c r="G34" s="21" t="n">
         <v>3</v>
@@ -7709,29 +9276,29 @@
         <v>69</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>625</v>
+        <v>741</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
-        <v>626</v>
+        <v>742</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>627</v>
+        <v>743</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>628</v>
+        <v>744</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>623</v>
+        <v>739</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>629</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G35" s="37" t="n">
+        <v>745</v>
+      </c>
+      <c r="F35" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G35" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("B5",Security!A:A,0))</f>
         <v>1</v>
       </c>
@@ -7739,29 +9306,29 @@
         <v>69</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>630</v>
+        <v>746</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>631</v>
+        <v>747</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>632</v>
+        <v>748</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>633</v>
+        <v>749</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>634</v>
+        <v>750</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>635</v>
-      </c>
-      <c r="F36" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G36" s="37" t="n">
+        <v>751</v>
+      </c>
+      <c r="F36" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G36" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("A1",Security!A:A,0))</f>
         <v>2</v>
       </c>
@@ -7769,29 +9336,29 @@
         <v>69</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>636</v>
+        <v>752</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>637</v>
+        <v>753</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>638</v>
+        <v>754</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>639</v>
+        <v>755</v>
       </c>
       <c r="D37" s="7" t="s">
+        <v>756</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="F37" s="54" t="s">
         <v>640</v>
       </c>
-      <c r="E37" s="7" t="s">
-        <v>641</v>
-      </c>
-      <c r="F37" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G37" s="37" t="n">
+      <c r="G37" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("A3",Security!A:A,0))+INDEX(Security!G:G,MATCH("A4",Security!A:A,0))</f>
         <v>2</v>
       </c>
@@ -7799,29 +9366,29 @@
         <v>69</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>642</v>
+        <v>758</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>643</v>
+        <v>759</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>644</v>
+        <v>760</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>645</v>
+        <v>761</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>646</v>
+        <v>762</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>647</v>
-      </c>
-      <c r="F38" s="38" t="s">
-        <v>493</v>
-      </c>
-      <c r="G38" s="37" t="n">
+        <v>763</v>
+      </c>
+      <c r="F38" s="53" t="s">
+        <v>609</v>
+      </c>
+      <c r="G38" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("B1",Security!A:A,0))+INDEX(Security!G:G,MATCH("B2",Security!A:A,0))</f>
         <v>2</v>
       </c>
@@ -7829,29 +9396,29 @@
         <v>69</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>648</v>
+        <v>764</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>649</v>
+        <v>765</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>650</v>
+        <v>766</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>651</v>
+        <v>767</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>652</v>
+        <v>768</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>653</v>
-      </c>
-      <c r="F39" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G39" s="37" t="n">
+        <v>769</v>
+      </c>
+      <c r="F39" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G39" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("A7",Security!A:A,0))</f>
         <v>3</v>
       </c>
@@ -7859,29 +9426,29 @@
         <v>69</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>654</v>
+        <v>770</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
-        <v>655</v>
+        <v>771</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>656</v>
+        <v>772</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>657</v>
+        <v>773</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>658</v>
+        <v>774</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>659</v>
-      </c>
-      <c r="F40" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G40" s="37" t="n">
+        <v>775</v>
+      </c>
+      <c r="F40" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G40" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("A6",Security!A:A,0))</f>
         <v>3</v>
       </c>
@@ -7889,61 +9456,61 @@
         <v>69</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>660</v>
+        <v>776</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="21" t="s">
-        <v>661</v>
+        <v>777</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>662</v>
+        <v>778</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>663</v>
+        <v>779</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>664</v>
+        <v>780</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>665</v>
-      </c>
-      <c r="F41" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G41" s="37" t="n">
+        <v>781</v>
+      </c>
+      <c r="F41" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G41" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("C2",Security!A:A,0))</f>
-        <v>1400</v>
+        <v>1209</v>
       </c>
       <c r="H41" s="21" t="s">
         <v>61</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>666</v>
+        <v>782</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="21" t="s">
-        <v>667</v>
+        <v>783</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>668</v>
+        <v>784</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>669</v>
+        <v>785</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>670</v>
+        <v>786</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>671</v>
-      </c>
-      <c r="F42" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G42" s="37" t="n">
+        <v>787</v>
+      </c>
+      <c r="F42" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G42" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("C1",Security!A:A,0))</f>
-        <v>1800</v>
+        <v>1993</v>
       </c>
       <c r="H42" s="21" t="s">
         <v>61</v>
@@ -7952,24 +9519,24 @@
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="21" t="s">
-        <v>672</v>
+        <v>788</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>673</v>
+        <v>789</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>674</v>
+        <v>790</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>675</v>
+        <v>791</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>676</v>
-      </c>
-      <c r="F43" s="39" t="s">
-        <v>524</v>
-      </c>
-      <c r="G43" s="37" t="n">
+        <v>792</v>
+      </c>
+      <c r="F43" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G43" s="36" t="n">
         <f aca="false">INDEX(Security!G:G,MATCH("B3",Security!A:A,0))</f>
         <v>1</v>
       </c>
@@ -7977,7 +9544,37 @@
         <v>69</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>677</v>
+        <v>793</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>797</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>798</v>
+      </c>
+      <c r="F44" s="54" t="s">
+        <v>640</v>
+      </c>
+      <c r="G44" s="36" t="n">
+        <f aca="false">INDEX(Security!G:G,MATCH("C5",Security!A:A,0))</f>
+        <v>1209</v>
+      </c>
+      <c r="H44" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="I44" s="8" t="s">
+        <v>799</v>
       </c>
     </row>
   </sheetData>
@@ -7991,7 +9588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8005,404 +9602,404 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="40" t="s">
-        <v>678</v>
+      <c r="B2" s="55" t="s">
+        <v>800</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="41" t="s">
-        <v>679</v>
-      </c>
-      <c r="C4" s="42"/>
+      <c r="B4" s="56" t="s">
+        <v>801</v>
+      </c>
+      <c r="C4" s="57"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="43" t="s">
-        <v>680</v>
+      <c r="B5" s="58" t="s">
+        <v>802</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>681</v>
+        <v>803</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="43" t="s">
-        <v>682</v>
+      <c r="B6" s="58" t="s">
+        <v>804</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>683</v>
+        <v>805</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="43" t="s">
-        <v>684</v>
+      <c r="B7" s="58" t="s">
+        <v>806</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>685</v>
+        <v>807</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="41" t="s">
-        <v>686</v>
-      </c>
-      <c r="C9" s="42"/>
+      <c r="B9" s="56" t="s">
+        <v>808</v>
+      </c>
+      <c r="C9" s="57"/>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="58" t="s">
         <v>76</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>687</v>
+        <v>809</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="58" t="s">
         <v>277</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>688</v>
+        <v>810</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="58" t="s">
         <v>60</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>689</v>
+        <v>811</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="58" t="s">
         <v>149</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>690</v>
+        <v>812</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="43" t="s">
-        <v>691</v>
+      <c r="B14" s="58" t="s">
+        <v>813</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>692</v>
+        <v>814</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="43" t="s">
-        <v>693</v>
+      <c r="B15" s="58" t="s">
+        <v>815</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>694</v>
+        <v>816</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="41" t="s">
-        <v>695</v>
-      </c>
-      <c r="C17" s="42"/>
+      <c r="B17" s="56" t="s">
+        <v>817</v>
+      </c>
+      <c r="C17" s="57"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="43" t="s">
-        <v>696</v>
+      <c r="B18" s="58" t="s">
+        <v>818</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>697</v>
+        <v>819</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="43" t="s">
-        <v>698</v>
+      <c r="B19" s="58" t="s">
+        <v>820</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>699</v>
+        <v>821</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="43" t="s">
-        <v>700</v>
+      <c r="B20" s="58" t="s">
+        <v>822</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>701</v>
+        <v>823</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="43" t="s">
-        <v>702</v>
+      <c r="B21" s="58" t="s">
+        <v>824</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>703</v>
+        <v>825</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="43" t="s">
-        <v>704</v>
+      <c r="B22" s="58" t="s">
+        <v>826</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>705</v>
+        <v>827</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="43" t="s">
-        <v>706</v>
+      <c r="B23" s="58" t="s">
+        <v>828</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>707</v>
+        <v>829</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="43" t="s">
-        <v>708</v>
+      <c r="B24" s="58" t="s">
+        <v>830</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>709</v>
+        <v>831</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="43" t="s">
-        <v>710</v>
+      <c r="B25" s="58" t="s">
+        <v>832</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>711</v>
+        <v>833</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="43" t="s">
-        <v>712</v>
+      <c r="B26" s="58" t="s">
+        <v>834</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>713</v>
+        <v>835</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="43" t="s">
-        <v>714</v>
+      <c r="B27" s="58" t="s">
+        <v>836</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>715</v>
+        <v>837</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="43" t="s">
-        <v>716</v>
+      <c r="B28" s="58" t="s">
+        <v>838</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>717</v>
+        <v>839</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="41" t="s">
-        <v>718</v>
-      </c>
-      <c r="C30" s="42"/>
+      <c r="B30" s="56" t="s">
+        <v>840</v>
+      </c>
+      <c r="C30" s="57"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="43" t="s">
-        <v>719</v>
+      <c r="B31" s="58" t="s">
+        <v>841</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>720</v>
+        <v>842</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="43" t="s">
-        <v>721</v>
+      <c r="B32" s="58" t="s">
+        <v>843</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>722</v>
+        <v>844</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="43" t="s">
-        <v>723</v>
+      <c r="B33" s="58" t="s">
+        <v>845</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>724</v>
+        <v>846</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="43" t="s">
-        <v>725</v>
+      <c r="B34" s="58" t="s">
+        <v>847</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>726</v>
+        <v>848</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="43" t="s">
-        <v>727</v>
+      <c r="B35" s="58" t="s">
+        <v>849</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>728</v>
+        <v>850</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="43" t="s">
-        <v>729</v>
+      <c r="B36" s="58" t="s">
+        <v>851</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>730</v>
+        <v>852</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="43" t="s">
-        <v>731</v>
+      <c r="B37" s="58" t="s">
+        <v>853</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>732</v>
+        <v>854</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="43" t="s">
-        <v>733</v>
+      <c r="B38" s="58" t="s">
+        <v>855</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>734</v>
+        <v>856</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="41" t="s">
-        <v>735</v>
-      </c>
-      <c r="C40" s="42"/>
+      <c r="B40" s="56" t="s">
+        <v>857</v>
+      </c>
+      <c r="C40" s="57"/>
     </row>
     <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="43" t="s">
-        <v>736</v>
+      <c r="B41" s="58" t="s">
+        <v>858</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>737</v>
+        <v>859</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="43" t="s">
-        <v>738</v>
+      <c r="B42" s="58" t="s">
+        <v>860</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>739</v>
+        <v>861</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="43" t="s">
-        <v>740</v>
+      <c r="B43" s="58" t="s">
+        <v>862</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>741</v>
+        <v>863</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="43" t="s">
-        <v>742</v>
+      <c r="B44" s="58" t="s">
+        <v>864</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>743</v>
+        <v>865</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="43" t="s">
-        <v>744</v>
+      <c r="B45" s="58" t="s">
+        <v>866</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>745</v>
+        <v>867</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="43" t="s">
-        <v>746</v>
+      <c r="B46" s="58" t="s">
+        <v>868</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>747</v>
+        <v>869</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="43" t="s">
-        <v>748</v>
+      <c r="B47" s="58" t="s">
+        <v>870</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>749</v>
+        <v>871</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="43" t="s">
-        <v>750</v>
+      <c r="B48" s="58" t="s">
+        <v>872</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>751</v>
+        <v>873</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="43" t="s">
-        <v>752</v>
+      <c r="B49" s="58" t="s">
+        <v>874</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>753</v>
+        <v>875</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="43" t="s">
-        <v>754</v>
+      <c r="B50" s="58" t="s">
+        <v>876</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>755</v>
+        <v>877</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="43" t="s">
-        <v>756</v>
+      <c r="B51" s="58" t="s">
+        <v>878</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>757</v>
+        <v>879</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="43" t="s">
-        <v>758</v>
+      <c r="B52" s="58" t="s">
+        <v>880</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>759</v>
+        <v>881</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="43" t="s">
-        <v>760</v>
+      <c r="B53" s="58" t="s">
+        <v>882</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>761</v>
+        <v>883</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B54" s="43" t="s">
-        <v>762</v>
+      <c r="B54" s="58" t="s">
+        <v>884</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>763</v>
+        <v>885</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="41" t="s">
-        <v>764</v>
-      </c>
-      <c r="C56" s="42"/>
+      <c r="B56" s="56" t="s">
+        <v>886</v>
+      </c>
+      <c r="C56" s="57"/>
     </row>
     <row r="57" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="43" t="s">
-        <v>765</v>
+      <c r="B57" s="58" t="s">
+        <v>887</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>766</v>
+        <v>888</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="43" t="s">
-        <v>767</v>
+      <c r="B58" s="58" t="s">
+        <v>889</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>768</v>
+        <v>890</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B59" s="43" t="s">
-        <v>769</v>
+      <c r="B59" s="58" t="s">
+        <v>891</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>770</v>
+        <v>892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>